<commit_message>
Did validation rules on DB, Updated Visual Diary, Updated Data Dictionary
</commit_message>
<xml_diff>
--- a/L2DTS - Data Dictionary.xlsx
+++ b/L2DTS - Data Dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://longbaycollege-my.sharepoint.com/personal/23029_lbc_school_nz/Documents/2026/L2DTS/Term 1/91892 - DTS Access DB Internal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="8_{3B400382-AA91-4064-9C8A-A9E72E6D8857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BC8B7F9-C980-48A7-86CB-F5C21E6151BB}"/>
+  <xr:revisionPtr revIDLastSave="204" documentId="8_{3B400382-AA91-4064-9C8A-A9E72E6D8857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0255706B-B815-463D-96E5-211371853EC1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{848A3F43-A1B8-40D4-935E-C2C61ED1AC88}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="91">
   <si>
     <t>Stock Table</t>
   </si>
@@ -306,6 +306,9 @@
   </si>
   <si>
     <t>The Date of the Order Placed</t>
+  </si>
+  <si>
+    <t>No Numbers</t>
   </si>
 </sst>
 </file>
@@ -951,13 +954,13 @@
   <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="59.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.5546875" style="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.88671875" style="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="26.4" thickTop="1" x14ac:dyDescent="0.5">
@@ -1174,7 +1177,9 @@
       <c r="C14" s="2">
         <v>255</v>
       </c>
-      <c r="D14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="E14" s="2" t="s">
         <v>63</v>
       </c>
@@ -1193,7 +1198,9 @@
       <c r="C15" s="2">
         <v>255</v>
       </c>
-      <c r="D15" s="2"/>
+      <c r="D15" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="E15" s="2" t="s">
         <v>64</v>
       </c>
@@ -1334,7 +1341,9 @@
       <c r="C24" s="3">
         <v>255</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="E24" s="3" t="s">
         <v>61</v>
       </c>
@@ -1353,7 +1362,9 @@
       <c r="C25" s="3">
         <v>255</v>
       </c>
-      <c r="D25" s="3"/>
+      <c r="D25" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="E25" s="3" t="s">
         <v>62</v>
       </c>

</xml_diff>